<commit_message>
Updated objectives and metrics table
</commit_message>
<xml_diff>
--- a/wr_sdm/documentation/objectives_metrics_v2.xlsx
+++ b/wr_sdm/documentation/objectives_metrics_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorg629193-my.sharepoint.com/personal/cpien_flowwest_com/Documents/Documents/Github/shasta-sdm/winterRunDSM/wr_sdm/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="135" documentId="8_{A967383E-92E9-4775-8C6E-A5264BA50E34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC276285-1E99-4EEB-BAB2-F328C6295932}"/>
+  <xr:revisionPtr revIDLastSave="138" documentId="8_{A967383E-92E9-4775-8C6E-A5264BA50E34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6225A595-C738-4AB4-935E-DA177EEC9B66}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{E83A208E-A424-474B-8313-B4DC6EABBEEC}"/>
+    <workbookView xWindow="-28920" yWindow="-4320" windowWidth="29040" windowHeight="15720" xr2:uid="{E83A208E-A424-474B-8313-B4DC6EABBEEC}"/>
   </bookViews>
   <sheets>
     <sheet name="objectives_metrics" sheetId="1" r:id="rId1"/>
@@ -56,9 +56,6 @@
     <t>mean_spawners</t>
   </si>
   <si>
-    <t>total_declines</t>
-  </si>
-  <si>
     <t>max_decline</t>
   </si>
   <si>
@@ -220,6 +217,9 @@
   </si>
   <si>
     <t>Estimated as the number of years with a 3-year population decline (based on total spawners across watersheds) of an order of magnitude or more.  The number of such 3-year catastrophic decline "events" over the 20-year modeling period is identified and reported.</t>
+  </si>
+  <si>
+    <t>cat_decline</t>
   </si>
 </sst>
 </file>
@@ -1173,10 +1173,10 @@
         <v>3</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -1190,13 +1190,13 @@
         <v>6</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -1207,16 +1207,16 @@
         <v>5</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:6" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -1230,13 +1230,13 @@
         <v>7</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -1247,176 +1247,176 @@
         <v>5</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>8</v>
+        <v>54</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="D6" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:6" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>10</v>
-      </c>
       <c r="C7" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>10</v>
-      </c>
       <c r="C8" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="D9" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="D10" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>19</v>
-      </c>
       <c r="C11" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>19</v>
-      </c>
       <c r="C12" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:6" s="2" customFormat="1" ht="135" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>19</v>
-      </c>
       <c r="C13" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
modified to add phos to diversity
</commit_message>
<xml_diff>
--- a/wr_sdm/documentation/objectives_metrics_v2.xlsx
+++ b/wr_sdm/documentation/objectives_metrics_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorg629193-my.sharepoint.com/personal/cpien_flowwest_com/Documents/Documents/Github/shasta-sdm/winterRunDSM/wr_sdm/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="140" documentId="8_{A967383E-92E9-4775-8C6E-A5264BA50E34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7735542-924B-42F4-861B-7A3CD11C2EF3}"/>
+  <xr:revisionPtr revIDLastSave="146" documentId="8_{A967383E-92E9-4775-8C6E-A5264BA50E34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D483BC2-222D-4AAE-AE38-8C99CB564B13}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-4320" windowWidth="29040" windowHeight="15720" xr2:uid="{E83A208E-A424-474B-8313-B4DC6EABBEEC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E83A208E-A424-474B-8313-B4DC6EABBEEC}"/>
   </bookViews>
   <sheets>
     <sheet name="objectives_metrics" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="56">
   <si>
     <t>objective</t>
   </si>
@@ -220,6 +220,9 @@
   </si>
   <si>
     <t>cat_decline</t>
+  </si>
+  <si>
+    <t>mean_phos_d</t>
   </si>
 </sst>
 </file>
@@ -1148,7 +1151,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8836ECF4-9848-4446-86BB-5107A1A11EC0}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.42578125" bestFit="1" customWidth="1"/>
@@ -1341,25 +1344,25 @@
     </row>
     <row r="10" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>19</v>
+        <v>55</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>49</v>
+        <v>35</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>17</v>
       </c>
@@ -1367,16 +1370,16 @@
         <v>18</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>26</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
@@ -1387,19 +1390,19 @@
         <v>18</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>26</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:6" s="2" customFormat="1" ht="135" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>17</v>
       </c>
@@ -1407,15 +1410,35 @@
         <v>18</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="F13" s="9" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" s="2" customFormat="1" ht="135" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F14" s="10" t="s">
         <v>52</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated the names of the metrics used for number of populations metrics
</commit_message>
<xml_diff>
--- a/wr_sdm/documentation/objectives_metrics_v2.xlsx
+++ b/wr_sdm/documentation/objectives_metrics_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorg629193-my.sharepoint.com/personal/cpien_flowwest_com/Documents/Documents/Github/shasta-sdm/winterRunDSM/wr_sdm/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="192" documentId="8_{A967383E-92E9-4775-8C6E-A5264BA50E34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4F0A9F80-B6C6-4868-816B-527268C4710E}"/>
+  <xr:revisionPtr revIDLastSave="208" documentId="8_{A967383E-92E9-4775-8C6E-A5264BA50E34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4ECA8193-DCCA-47DF-9AD4-E9CC1415BAA4}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E83A208E-A424-474B-8313-B4DC6EABBEEC}"/>
+    <workbookView xWindow="-28920" yWindow="-4320" windowWidth="29040" windowHeight="15720" xr2:uid="{E83A208E-A424-474B-8313-B4DC6EABBEEC}"/>
   </bookViews>
   <sheets>
     <sheet name="objectives_metrics" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="88">
   <si>
     <t>objective</t>
   </si>
@@ -119,18 +119,12 @@
     <t>Proportion of total suitable rearing habitat that is in tributaries</t>
   </si>
   <si>
-    <t>mean_juv_rear_trib</t>
-  </si>
-  <si>
     <t>Number of tributaries above Shasta Dam with accessible spawning and rearing habitat</t>
   </si>
   <si>
     <t>Number of independent populations</t>
   </si>
   <si>
-    <t>num_trib</t>
-  </si>
-  <si>
     <t>Represents an interest in increasing WRCS abundance across the watershed.</t>
   </si>
   <si>
@@ -180,9 +174,6 @@
   </si>
   <si>
     <t>Spawner outputs are filtered to include only tributary spawners and summed annually across tributaries, then summarized by  the  20-year average value of total tributary spawners. Tributaries considered are the McCloud River, Little Sacramento River, and Battle Creek.</t>
-  </si>
-  <si>
-    <t>Available annual rearing habitat in tributaries is summed, then divided by the annual total amount of available rearing habitat in the watershed. Results are then summarized to show the  20-year average value of proportion of suitable rearing habitat found in tributaries. Tributaries considered are the McCloud River, Little Sacramento River, and Battle Creek.</t>
   </si>
   <si>
     <t>Actions including trap and haul and removal of barriers to above Shasta habitat increase habitat available to WRCS above Shasta in the WRCS model. If both rearing habitat and spawning habitat values are greater than 0, the tributary is considered to be accessible. Tributaries considered are the McCloud River and Little Sacramento River. This value is reported as a count: 0, 1, or 2.</t>
@@ -255,9 +246,6 @@
     <t>Ability of WRCS to live their natural life-cycle</t>
   </si>
   <si>
-    <t xml:space="preserve">Increases human interventions (e.g. hatchery, transport, handling, or infrastructure operations) </t>
-  </si>
-  <si>
     <t>Change in human intervention</t>
   </si>
   <si>
@@ -307,6 +295,30 @@
   </si>
   <si>
     <t>Average pHOS (abundance)</t>
+  </si>
+  <si>
+    <t>0 for no effect on Fall-Run Chinook Salmon, 1, 2, 3, 4.</t>
+  </si>
+  <si>
+    <t>Negative if actions increase human interventions (e.g. hatchery, transport, handling, or infrastructure operations), positive if actions decrease human interventions, neutral if neither.</t>
+  </si>
+  <si>
+    <t>0 for no effect on other list species, 1, 2, 3, 4.</t>
+  </si>
+  <si>
+    <t>Costs estimated based on participant input, then scaled.</t>
+  </si>
+  <si>
+    <t>Constructed scale: 1 for &lt; 1 year, 2 for 1-5 years, 3 for 5-10 years, 4 for 10+ years</t>
+  </si>
+  <si>
+    <t>hab_access</t>
+  </si>
+  <si>
+    <t>Available annual rearing habitat in tributaries is summed, then divided by the annual total amount of available rearing habitat in the Upper Sacramento and tributaries. Results are then summarized to show the  20-year average value of proportion of suitable rearing habitat found in tributaries. Tributaries considered are the McCloud River, Little Sacramento River, and Battle Creek.</t>
+  </si>
+  <si>
+    <t>mean_rear_prop</t>
   </si>
 </sst>
 </file>
@@ -767,16 +779,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -825,7 +837,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -834,22 +846,19 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -859,6 +868,13 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1242,393 +1258,408 @@
     <col min="2" max="2" width="38" style="1" customWidth="1"/>
     <col min="3" max="3" width="29.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="43.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="43.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="43.7109375" style="3" customWidth="1"/>
     <col min="6" max="6" width="73.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="9" t="s">
+      <c r="E6" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" s="2" customFormat="1" ht="135" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="F20" s="12" t="s">
         <v>83</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F8" s="10" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F12" s="9" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F13" s="9" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" s="2" customFormat="1" ht="135" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F14" s="10" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C15" t="s">
-        <v>55</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="F15" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="C18" t="s">
-        <v>58</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="C19" t="s">
-        <v>59</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="C20" t="s">
-        <v>60</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated language to match report
</commit_message>
<xml_diff>
--- a/wr_sdm/documentation/objectives_metrics_v2.xlsx
+++ b/wr_sdm/documentation/objectives_metrics_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorg629193-my.sharepoint.com/personal/cpien_flowwest_com/Documents/Documents/Github/shasta-sdm/winterRunDSM/wr_sdm/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="208" documentId="8_{A967383E-92E9-4775-8C6E-A5264BA50E34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4ECA8193-DCCA-47DF-9AD4-E9CC1415BAA4}"/>
+  <xr:revisionPtr revIDLastSave="211" documentId="8_{A967383E-92E9-4775-8C6E-A5264BA50E34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4305E646-7385-4DC7-8A2C-4EC0479FF5B2}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-4320" windowWidth="29040" windowHeight="15720" xr2:uid="{E83A208E-A424-474B-8313-B4DC6EABBEEC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E83A208E-A424-474B-8313-B4DC6EABBEEC}"/>
   </bookViews>
   <sheets>
     <sheet name="objectives_metrics" sheetId="1" r:id="rId1"/>
@@ -152,16 +152,7 @@
     <t>Average annual number of adults spawning in tributaries (Battle Creek and Above Shasta Dam)</t>
   </si>
   <si>
-    <t xml:space="preserve">Model estimates the number of adult spawning salmonids in each tributary, for each year of the 20-year simulation. Spawners for each watershed are summed annually, then those totals are averaged across the 20 years to yeield the average value of total spawners. </t>
-  </si>
-  <si>
     <t>Proportion of hatchery spawners (pHOS) is estimated by dividing total hatchery-origin spawner (considering all watersheds/tributaries) by total spawners, for each year of the 20-year simulation.  Those pHOS values are then averaged over the 20 years and that value is reported for this metric.</t>
-  </si>
-  <si>
-    <t>Year over year decline in number of total spawners is calculated for each year of the modeling period (20 years). The longest run of consecutive years with greater than or equal to 10% decline is identfied and reported.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimated with models as the annual number of juveniles exiting the Upper Sacramento at Red Bluff prior to undergoing rearing, outmigration, and growth. Model results are summarized withone 20-year average value of number of juveniles. </t>
   </si>
   <si>
     <t xml:space="preserve">Estimated with models as the annual number of smolts (larger juveniles) reaching Chipps Island. Model results are summarized with the 20-year average value of number of smolts. </t>
@@ -319,6 +310,15 @@
   </si>
   <si>
     <t>mean_rear_prop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model estimates the number of adult spawning salmonids in each tributary, for each year of the 20-year simulation. Spawners for each watershed are summed annually, then those totals are averaged across the 20 years to yield the average value of total spawners. </t>
+  </si>
+  <si>
+    <t>Year over year decline in number of total spawners is calculated for each year of the modeling period (20 years). The longest run of consecutive years with greater than or equal to 10% decline is identified and reported.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimated with models as the annual number of juveniles exiting the Upper Sacramento at Red Bluff prior to undergoing rearing, outmigration, and growth. Model results are summarized with one 20-year average value of number of juveniles. </t>
   </si>
 </sst>
 </file>
@@ -1299,7 +1299,7 @@
         <v>30</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>39</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -1313,13 +1313,13 @@
         <v>16</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E3" s="9" t="s">
         <v>31</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:6" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -1339,7 +1339,7 @@
         <v>30</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>41</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -1350,7 +1350,7 @@
         <v>5</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>23</v>
@@ -1359,7 +1359,7 @@
         <v>30</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -1379,7 +1379,7 @@
         <v>25</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>42</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" spans="1:6" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -1399,7 +1399,7 @@
         <v>25</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
@@ -1419,7 +1419,7 @@
         <v>25</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -1439,7 +1439,7 @@
         <v>24</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -1450,16 +1450,16 @@
         <v>14</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>24</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -1479,7 +1479,7 @@
         <v>26</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
@@ -1490,7 +1490,7 @@
         <v>18</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D12" s="8" t="s">
         <v>27</v>
@@ -1499,7 +1499,7 @@
         <v>26</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
@@ -1510,7 +1510,7 @@
         <v>18</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>28</v>
@@ -1519,7 +1519,7 @@
         <v>26</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:6" s="2" customFormat="1" ht="135" x14ac:dyDescent="0.25">
@@ -1539,127 +1539,127 @@
         <v>26</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="F16" s="12" t="s">
         <v>77</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="D16" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="F16" s="12" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D19" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="E19" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="E19" s="11" t="s">
-        <v>71</v>
-      </c>
       <c r="F19" s="12" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated some of the text for metrics
</commit_message>
<xml_diff>
--- a/wr_sdm/documentation/objectives_metrics_v2.xlsx
+++ b/wr_sdm/documentation/objectives_metrics_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorg629193-my.sharepoint.com/personal/cpien_flowwest_com/Documents/Documents/Github/shasta-sdm/winterRunDSM/wr_sdm/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="211" documentId="8_{A967383E-92E9-4775-8C6E-A5264BA50E34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4305E646-7385-4DC7-8A2C-4EC0479FF5B2}"/>
+  <xr:revisionPtr revIDLastSave="212" documentId="8_{A967383E-92E9-4775-8C6E-A5264BA50E34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5E378A30-4D8A-4D19-BC3B-DC9B4A9C0E32}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E83A208E-A424-474B-8313-B4DC6EABBEEC}"/>
   </bookViews>
@@ -152,52 +152,6 @@
     <t>Average annual number of adults spawning in tributaries (Battle Creek and Above Shasta Dam)</t>
   </si>
   <si>
-    <t>Proportion of hatchery spawners (pHOS) is estimated by dividing total hatchery-origin spawner (considering all watersheds/tributaries) by total spawners, for each year of the 20-year simulation.  Those pHOS values are then averaged over the 20 years and that value is reported for this metric.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimated with models as the annual number of smolts (larger juveniles) reaching Chipps Island. Model results are summarized with the 20-year average value of number of smolts. </t>
-  </si>
-  <si>
-    <t>Cohort Replacement Rate (CRR) is estimated with models as the adult natural origin return ratio in each tributary, tracked for 20 years. CRR is calculated annually as the total number of natural origin adult returns across watersheds in year X+3 divided by the number of total spawners across watersheds in year X. The 20-year average value is reported.</t>
-  </si>
-  <si>
-    <t>Salmonid models can be used to estimate the annual variation of size (small, medium, large, very large) in juveniles at ocean entry. Size distribution of juveniles is summarized in a single metric by using a Shannon diversity index, calculated for each year.  The 20-year average of the annual value is reported.</t>
-  </si>
-  <si>
-    <t>Spawner outputs are filtered to include only tributary spawners and summed annually across tributaries, then summarized by  the  20-year average value of total tributary spawners. Tributaries considered are the McCloud River, Little Sacramento River, and Battle Creek.</t>
-  </si>
-  <si>
-    <t>Actions including trap and haul and removal of barriers to above Shasta habitat increase habitat available to WRCS above Shasta in the WRCS model. If both rearing habitat and spawning habitat values are greater than 0, the tributary is considered to be accessible. Tributaries considered are the McCloud River and Little Sacramento River. This value is reported as a count: 0, 1, or 2.</t>
-  </si>
-  <si>
-    <r>
-      <t>Watershed-specific estimates from models can be used to calculate the number of independent viable populations of WRCS. Independent populations are defined as those meeting the following criteria: greater than 500 spawners, pHOS less than 5%, CRR &gt; 1, spawner increase &gt; 1. If a population met the thresholds for the</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> last 3 years of the modeling period that have values for those metrics</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF1C1D1F"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, this was considered an independent population. Watersheds considered are the McCloud River, Little Sacramento River, Battle Creek, and the Upper Sacramento River. pHOS and CRR values in the Upper Sacramento River and above Shasta tributaries will be the same.</t>
-    </r>
-  </si>
-  <si>
-    <t>Estimated as the number of years with a 3-year population decline (based on total spawners across watersheds) of an order of magnitude or more.  The number of such 3-year catastrophic decline "events" over the 20-year modeling period is identified and reported.</t>
-  </si>
-  <si>
     <t>cat_decline</t>
   </si>
   <si>
@@ -306,26 +260,50 @@
     <t>hab_access</t>
   </si>
   <si>
-    <t>Available annual rearing habitat in tributaries is summed, then divided by the annual total amount of available rearing habitat in the Upper Sacramento and tributaries. Results are then summarized to show the  20-year average value of proportion of suitable rearing habitat found in tributaries. Tributaries considered are the McCloud River, Little Sacramento River, and Battle Creek.</t>
-  </si>
-  <si>
     <t>mean_rear_prop</t>
   </si>
   <si>
-    <t xml:space="preserve">Model estimates the number of adult spawning salmonids in each tributary, for each year of the 20-year simulation. Spawners for each watershed are summed annually, then those totals are averaged across the 20 years to yield the average value of total spawners. </t>
-  </si>
-  <si>
     <t>Year over year decline in number of total spawners is calculated for each year of the modeling period (20 years). The longest run of consecutive years with greater than or equal to 10% decline is identified and reported.</t>
   </si>
   <si>
-    <t xml:space="preserve">Estimated with models as the annual number of juveniles exiting the Upper Sacramento at Red Bluff prior to undergoing rearing, outmigration, and growth. Model results are summarized with one 20-year average value of number of juveniles. </t>
+    <t>Model estimates the number of adult spawning salmonids in each tributary, for each year of the 20-year simulation. Spawners for each watershed unit were summed annually, then those totals were averaged across the 20 years to yield the average value of total spawners.</t>
+  </si>
+  <si>
+    <t>Proportion of hatchery-origin spawners (pHOS) was estimated by dividing total hatchery-origin spawners (considering all watersheds units) by total spawners, for each year of the 20-year simulation. Those pHOS values were then averaged across the 20 years to yield the average pHOS.</t>
+  </si>
+  <si>
+    <t>Estimated as the number of years with a 3-year population decline (based on total spawners across watershed units) of an order of magnitude or more. The number of such 3-year catastrophic decline "events" over the 20-year modeling period is identified and reported.</t>
+  </si>
+  <si>
+    <t>Estimated with models as the annual number of juveniles exiting the Upper Sacramento at Red Bluff prior to undergoing rearing, outmigration, and growth. Model results were summarized with one 20-year average value of number of juveniles.</t>
+  </si>
+  <si>
+    <t>Estimated with models as the annual number of smolts (larger juveniles) reaching Chipps Island. Model results were summarized with the 20-year average value of number of smolts.</t>
+  </si>
+  <si>
+    <t>Cohort Replacement Rate (CRR) is estimated with models as the adult natural origin return ratio in each tributary, tracked for 20 years. CRR is calculated annually as the total number of natural-origin adult returns in year X+3 divided by the number of total spawners in year X. Natural-origin and total spawners were each summed across watershed units annually and the 20-year average value is reported.</t>
+  </si>
+  <si>
+    <t>Salmonid models can be used to estimate the annual variation of size (small, medium, large, very large) in juveniles at ocean entry. Size distribution of juveniles is summarized in a single metric by using a Shannon diversity index, calculated for each year. The 20-year average of the annual value is reported.</t>
+  </si>
+  <si>
+    <t>Spawners above dam model outputs were summed annually with Battle Creek returns, then summarized by the 20-year average value of total tributary spawners.</t>
+  </si>
+  <si>
+    <t>Available annual rearing habitat in tributaries was calculated for each portfolio by summing instream and floodplain habitat in each tributary (McCloud, Little Sacramento, Battle Creek) for each year and dividing by the total rearing habitat across tributaries and the Upper Sacramento mainstem. Results were then summarized to show the 20-year average value of proportion of suitable rearing habitat found in tributaries.</t>
+  </si>
+  <si>
+    <t>Actions including trap and haul and removal of barriers to above Shasta habitat increase habitat available to WRCS above Shasta in the WRCS model. Based on the method described above, if both rearing habitat and spawning habitat proportions were greater than 0, the tributary was considered to be accessible. Tributaries considered were the McCloud River and Little Sacramento River. This value is reported as a count: 0 (no tributaries accessible), 1 (either McCloud or Little Sacramento accessible), or 2 (both McCloud and Little Sacramento accessible).</t>
+  </si>
+  <si>
+    <t>Watershed-specific estimates from models can be used to calculate the number of independent viable populations of WRCS. Independent populations were defined as those meeting the following criteria: greater than 500 spawners, pHOS less than 5%, CRR &gt; 1, spawner increase &gt; 1. If a population met the thresholds for the last 3 years of the modeling period that have values for those metrics, this was considered an independent population. Watersheds considered were the McCloud River, Little Sacramento River, Battle Creek, and the Upper Sacramento River below Shasta. Spawners for the Upper Sacramento River watershed unit were estimated by using the proportion of habitat available in each of the watersheds (Upper Sacramento mainstem, McCloud, Little Sacramento) for each portfolio multiplied by the total returns in the Upper Sacramento watershed.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -480,6 +458,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="33">
     <fill>
@@ -662,7 +646,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -792,6 +776,34 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -837,7 +849,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -875,6 +887,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1262,7 +1280,7 @@
     <col min="6" max="6" width="73.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1282,7 +1300,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" s="2" customFormat="1" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>4</v>
       </c>
@@ -1298,11 +1316,11 @@
       <c r="E2" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="F2" s="8" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="F2" s="14" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" s="2" customFormat="1" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
@@ -1313,16 +1331,16 @@
         <v>16</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="E3" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="F3" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="F3" s="15" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="2" customFormat="1" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>4</v>
       </c>
@@ -1338,11 +1356,11 @@
       <c r="E4" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="F4" s="8" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="F4" s="15" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="2" customFormat="1" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>4</v>
       </c>
@@ -1350,7 +1368,7 @@
         <v>5</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>23</v>
@@ -1358,11 +1376,11 @@
       <c r="E5" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="8" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="F5" s="15" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="2" customFormat="1" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>8</v>
       </c>
@@ -1378,11 +1396,11 @@
       <c r="E6" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="8" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" s="2" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="F6" s="15" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="2" customFormat="1" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>8</v>
       </c>
@@ -1398,11 +1416,11 @@
       <c r="E7" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="F7" s="8" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+      <c r="F7" s="15" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="2" customFormat="1" ht="72" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>8</v>
       </c>
@@ -1418,11 +1436,11 @@
       <c r="E8" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="F8" s="9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="F8" s="15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="2" customFormat="1" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>13</v>
       </c>
@@ -1438,11 +1456,11 @@
       <c r="E9" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="F9" s="8" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="F9" s="15" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="2" customFormat="1" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>13</v>
       </c>
@@ -1450,19 +1468,19 @@
         <v>14</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="F10" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" s="2" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="F10" s="15" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" s="2" customFormat="1" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>17</v>
       </c>
@@ -1478,11 +1496,11 @@
       <c r="E11" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="8" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+      <c r="F11" s="15" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" s="2" customFormat="1" ht="86.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
         <v>17</v>
       </c>
@@ -1490,7 +1508,7 @@
         <v>18</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="D12" s="8" t="s">
         <v>27</v>
@@ -1498,11 +1516,11 @@
       <c r="E12" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="F12" s="8" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" s="2" customFormat="1" ht="75" x14ac:dyDescent="0.25">
+      <c r="F12" s="15" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="2" customFormat="1" ht="100.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>17</v>
       </c>
@@ -1510,7 +1528,7 @@
         <v>18</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>28</v>
@@ -1518,11 +1536,11 @@
       <c r="E13" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="F13" s="8" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" s="2" customFormat="1" ht="135" x14ac:dyDescent="0.25">
+      <c r="F13" s="15" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" s="2" customFormat="1" ht="157.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>17</v>
       </c>
@@ -1538,128 +1556,128 @@
       <c r="E14" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="F14" s="9" t="s">
-        <v>45</v>
+      <c r="F14" s="15" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="E15" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="F15" s="13" t="s">
         <v>70</v>
-      </c>
-      <c r="F15" s="13" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="E16" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="F16" s="12" t="s">
         <v>69</v>
-      </c>
-      <c r="F16" s="12" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>